<commit_message>
Center and top-align scheduling Excel cell text.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CALE-V5-main/docs/school/programacion-hoy-ejemplo.xlsx
+++ b/CALE-V5-main/docs/school/programacion-hoy-ejemplo.xlsx
@@ -34,7 +34,7 @@
     <x:t>Generado (Colombia)</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-28 10:48</x:t>
+    <x:t>2026-10-28 10:57</x:t>
   </x:si>
   <x:si>
     <x:t>Resumen</x:t>
@@ -109,7 +109,7 @@
     <x:t>Scheduled</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-27 16:48</x:t>
+    <x:t>2026-10-27 16:57</x:t>
   </x:si>
   <x:si>
     <x:t>Ana María Pérez López</x:t>
@@ -127,7 +127,7 @@
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>2026-10-27 22:48</x:t>
+    <x:t>2026-10-27 22:57</x:t>
   </x:si>
   <x:si>
     <x:t>Carlos Andrés Ruiz</x:t>
@@ -139,7 +139,7 @@
     <x:t>3109876543</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-28 04:48</x:t>
+    <x:t>2026-10-28 04:57</x:t>
   </x:si>
   <x:si>
     <x:t>Diana Sofía Vargas</x:t>
@@ -178,7 +178,7 @@
     <x:t>Pedro Castillo</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-27 04:48</x:t>
+    <x:t>2026-10-27 04:57</x:t>
   </x:si>
   <x:si>
     <x:t>Elena Patricia Mora</x:t>
@@ -190,7 +190,7 @@
     <x:t>3012223344</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-28 06:48</x:t>
+    <x:t>2026-10-28 06:57</x:t>
   </x:si>
   <x:si>
     <x:t>Felipe José Herrera</x:t>
@@ -214,7 +214,7 @@
     <x:t>Andrés Melo</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-26 18:48</x:t>
+    <x:t>2026-10-26 18:57</x:t>
   </x:si>
   <x:si>
     <x:t>Gabriel Eduardo Niño</x:t>
@@ -244,7 +244,7 @@
     <x:t>Past</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-26 08:48</x:t>
+    <x:t>2026-10-26 08:57</x:t>
   </x:si>
   <x:si>
     <x:t>Braynner Estudiante Demo</x:t>
@@ -583,68 +583,68 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
@@ -1044,132 +1044,132 @@
     <x:col min="14" max="14" width="16.996339" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:14" s="2" customFormat="1">
-      <x:c r="A1" s="3" t="s">
+    <x:row r="1" spans="1:14">
+      <x:c r="A1" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="s">
+      <x:c r="B1" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="s">
+      <x:c r="C1" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="s">
+      <x:c r="D1" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="s">
+      <x:c r="E1" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="s">
+      <x:c r="F1" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="s">
+      <x:c r="G1" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="s">
+      <x:c r="H1" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="s">
+      <x:c r="I1" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="s">
+      <x:c r="J1" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="s">
+      <x:c r="K1" s="2" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="s">
+      <x:c r="L1" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="s">
+      <x:c r="M1" s="2" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="N1" s="3" t="s">
+      <x:c r="N1" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:14">
-      <x:c r="A2" s="4" t="s">
+      <x:c r="A2" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="s">
+      <x:c r="B2" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="s">
+      <x:c r="C2" s="4" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="s">
+      <x:c r="D2" s="4" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="s">
+      <x:c r="E2" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F2" s="5">
+      <x:c r="F2" s="4">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="G2" s="5">
+      <x:c r="G2" s="4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H2" s="5">
+      <x:c r="H2" s="4">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="I2" s="5" t="s">
+      <x:c r="I2" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="J2" s="6" t="s">
+      <x:c r="J2" s="5" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="K2" s="6" t="s">
+      <x:c r="K2" s="5" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="L2" s="6" t="s">
+      <x:c r="L2" s="5" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="M2" s="6" t="s">
+      <x:c r="M2" s="5" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="N2" s="7" t="s">
+      <x:c r="N2" s="6" t="s">
         <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:14">
-      <x:c r="A3" s="8" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="I3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="J3" s="0" t="s">
+      <x:c r="A3" s="7" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="I3" s="8" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="J3" s="8" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="K3" s="0" t="s">
+      <x:c r="K3" s="8" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="L3" s="0" t="s">
+      <x:c r="L3" s="8" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="M3" s="0" t="s">
+      <x:c r="M3" s="8" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="N3" s="9" t="s">
@@ -1220,7 +1220,22 @@
         <x:v>44</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:14" ht="10" customHeight="1"/>
+    <x:row r="5" spans="1:14" ht="10" customHeight="1">
+      <x:c r="A5" s="8"/>
+      <x:c r="B5" s="8"/>
+      <x:c r="C5" s="8"/>
+      <x:c r="D5" s="8"/>
+      <x:c r="E5" s="8"/>
+      <x:c r="F5" s="8"/>
+      <x:c r="G5" s="8"/>
+      <x:c r="H5" s="8"/>
+      <x:c r="I5" s="8"/>
+      <x:c r="J5" s="8"/>
+      <x:c r="K5" s="8"/>
+      <x:c r="L5" s="8"/>
+      <x:c r="M5" s="8"/>
+      <x:c r="N5" s="8"/>
+    </x:row>
     <x:row r="6" spans="1:14">
       <x:c r="A6" s="13" t="s">
         <x:v>8</x:v>
@@ -1265,48 +1280,63 @@
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:14" ht="10" customHeight="1"/>
+    <x:row r="7" spans="1:14" ht="10" customHeight="1">
+      <x:c r="A7" s="8"/>
+      <x:c r="B7" s="8"/>
+      <x:c r="C7" s="8"/>
+      <x:c r="D7" s="8"/>
+      <x:c r="E7" s="8"/>
+      <x:c r="F7" s="8"/>
+      <x:c r="G7" s="8"/>
+      <x:c r="H7" s="8"/>
+      <x:c r="I7" s="8"/>
+      <x:c r="J7" s="8"/>
+      <x:c r="K7" s="8"/>
+      <x:c r="L7" s="8"/>
+      <x:c r="M7" s="8"/>
+      <x:c r="N7" s="8"/>
+    </x:row>
     <x:row r="8" spans="1:14">
-      <x:c r="A8" s="4" t="s">
+      <x:c r="A8" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="B8" s="4" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
+      <x:c r="C8" s="4" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="s">
+      <x:c r="D8" s="4" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="E8" s="5" t="s">
+      <x:c r="E8" s="4" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="F8" s="5">
+      <x:c r="F8" s="4">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="G8" s="5">
+      <x:c r="G8" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H8" s="5">
+      <x:c r="H8" s="4">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="I8" s="5" t="s">
+      <x:c r="I8" s="4" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="J8" s="6" t="s">
+      <x:c r="J8" s="5" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="K8" s="6" t="s">
+      <x:c r="K8" s="5" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="L8" s="6" t="s">
+      <x:c r="L8" s="5" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="M8" s="6" t="s">
+      <x:c r="M8" s="5" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="N8" s="7" t="s">
+      <x:c r="N8" s="6" t="s">
         <x:v>34</x:v>
       </x:c>
     </x:row>
@@ -1387,47 +1417,47 @@
     <x:col min="14" max="14" width="16.996339" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:14" s="2" customFormat="1">
-      <x:c r="A1" s="3" t="s">
+    <x:row r="1" spans="1:14">
+      <x:c r="A1" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="s">
+      <x:c r="B1" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="s">
+      <x:c r="C1" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="s">
+      <x:c r="D1" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="s">
+      <x:c r="E1" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="s">
+      <x:c r="F1" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="s">
+      <x:c r="G1" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="s">
+      <x:c r="H1" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="s">
+      <x:c r="I1" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="s">
+      <x:c r="J1" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="s">
+      <x:c r="K1" s="2" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="s">
+      <x:c r="L1" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="s">
+      <x:c r="M1" s="2" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="N1" s="3" t="s">
+      <x:c r="N1" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1475,7 +1505,22 @@
         <x:v>34</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:14" ht="10" customHeight="1"/>
+    <x:row r="3" spans="1:14" ht="10" customHeight="1">
+      <x:c r="A3" s="8"/>
+      <x:c r="B3" s="8"/>
+      <x:c r="C3" s="8"/>
+      <x:c r="D3" s="8"/>
+      <x:c r="E3" s="8"/>
+      <x:c r="F3" s="8"/>
+      <x:c r="G3" s="8"/>
+      <x:c r="H3" s="8"/>
+      <x:c r="I3" s="8"/>
+      <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
+      <x:c r="L3" s="8"/>
+      <x:c r="M3" s="8"/>
+      <x:c r="N3" s="8"/>
+    </x:row>
     <x:row r="4" spans="1:14">
       <x:c r="A4" s="13" t="s">
         <x:v>9</x:v>
@@ -1553,47 +1598,47 @@
     <x:col min="14" max="14" width="16.996339" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:14" s="2" customFormat="1">
-      <x:c r="A1" s="3" t="s">
+    <x:row r="1" spans="1:14">
+      <x:c r="A1" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="s">
+      <x:c r="B1" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="s">
+      <x:c r="C1" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="s">
+      <x:c r="D1" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="s">
+      <x:c r="E1" s="2" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="s">
+      <x:c r="F1" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="s">
+      <x:c r="G1" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="s">
+      <x:c r="H1" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="s">
+      <x:c r="I1" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="s">
+      <x:c r="J1" s="2" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="s">
+      <x:c r="K1" s="2" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="s">
+      <x:c r="L1" s="2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="s">
+      <x:c r="M1" s="2" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="N1" s="3" t="s">
+      <x:c r="N1" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1641,7 +1686,22 @@
         <x:v>79</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:14" ht="10" customHeight="1"/>
+    <x:row r="3" spans="1:14" ht="10" customHeight="1">
+      <x:c r="A3" s="8"/>
+      <x:c r="B3" s="8"/>
+      <x:c r="C3" s="8"/>
+      <x:c r="D3" s="8"/>
+      <x:c r="E3" s="8"/>
+      <x:c r="F3" s="8"/>
+      <x:c r="G3" s="8"/>
+      <x:c r="H3" s="8"/>
+      <x:c r="I3" s="8"/>
+      <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
+      <x:c r="L3" s="8"/>
+      <x:c r="M3" s="8"/>
+      <x:c r="N3" s="8"/>
+    </x:row>
     <x:row r="4" spans="1:14">
       <x:c r="A4" s="13" t="s">
         <x:v>72</x:v>
@@ -1686,7 +1746,22 @@
         <x:v>35</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:14" ht="10" customHeight="1"/>
+    <x:row r="5" spans="1:14" ht="10" customHeight="1">
+      <x:c r="A5" s="8"/>
+      <x:c r="B5" s="8"/>
+      <x:c r="C5" s="8"/>
+      <x:c r="D5" s="8"/>
+      <x:c r="E5" s="8"/>
+      <x:c r="F5" s="8"/>
+      <x:c r="G5" s="8"/>
+      <x:c r="H5" s="8"/>
+      <x:c r="I5" s="8"/>
+      <x:c r="J5" s="8"/>
+      <x:c r="K5" s="8"/>
+      <x:c r="L5" s="8"/>
+      <x:c r="M5" s="8"/>
+      <x:c r="N5" s="8"/>
+    </x:row>
     <x:row r="6" spans="1:14">
       <x:c r="A6" s="13" t="s">
         <x:v>72</x:v>

</xml_diff>